<commit_message>
Improve ingestion template descriptions
</commit_message>
<xml_diff>
--- a/Excel Templates/column-ingestion-template.xlsx
+++ b/Excel Templates/column-ingestion-template.xlsx
@@ -445,7 +445,7 @@
     </comment>
     <comment ref="A8" authorId="0" shapeId="0">
       <text>
-        <t>"y" = a blank lithology/strat_name/etc. cell copies the value from the unit above (type "none" to stop). Do not leave blank.
+        <t>"y" = a blank lithology/strat_name/etc. cell copies the value from the unit below it, so enter a value at the base of the interval it applies to (type "none" to stop). Do not leave blank.
 Format: y or n</t>
       </text>
     </comment>
@@ -601,8 +601,8 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>HEIGHT OF THE TOP of this unit. Fill it ONLY on the topmost unit of each column; every other top is taken from the b_pos of the unit above.
-Format: Number (metres), top unit only</t>
+        <t>HEIGHT OF THE TOP of this unit. Fill it ONLY on the topmost unit of each column, or on a unit below a gap; every other top is taken from the b_pos of the unit above. Or leave it blank and add an empty closing row above the top unit, with only col_id and b_pos.
+Format: Number (metres), top unit or below a gap</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -619,108 +619,8 @@
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Formation or member name, as named in Macrostrat. Fill strat_name, unit_name, or both: each unit needs at least one. If unit_name is blank, this becomes the unit's name.
-Format: Text</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>A local name for the unit (e.g. "upper carbonate"). Fill unit_name, strat_name, or both: each unit needs at least one. If both are filled, this is the unit's name.
-Format: Text</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Type of contact at the bottom of the unit.
-Format: Text, e.g. nonconformity, conformable</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>AGE AT THE BOTTOM of this unit, as a geologic time interval. Fill only at tie points (where you know the age); at least 2 per column. Ages in between are interpolated.
-Format: Macrostrat interval name (use the dropdown)</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>WHERE IN THAT INTERVAL the bottom falls: 0 = start (oldest) of the interval, 0.5 = middle, 1 = end (youngest). A blank counts as 0, so give a best guess.
-Format: Number from 0 to 1</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t>Age at the top. Usually blank: it is taken from the unit above. Fill only on the top unit if its age is known.
-Format: Interval name, or blank</t>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <t>Where in t_int the top falls (0-1). Usually blank.
-Format: Number 0-1, or blank</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <t>Why you chose each age tie point and proportion.
-Format: Text</t>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional label linking to the facies tab. Not read on upload: still fill lithology.
-Format: Text, e.g. F1</t>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <t>Generalizations, gaps or covered intervals, anything a reader should know.
-Format: Text</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Macrostrat</author>
-  </authors>
-  <commentList>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>Which column this unit belongs to.
-Format: A col_id from the columns tab</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>Leave blank if the column is one continuous section. Use a new ID only where the age model breaks (e.g. a fault).
-Format: Text, or blank</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>HEIGHT OF THE BOTTOM of this unit, in metres measured up from the base of the column (base = 0). Every unit needs one.
-Format: Number (metres)</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>HEIGHT OF THE TOP of this unit. Fill it ONLY on the topmost unit of each column; every other top is taken from the b_pos of the unit above.
-Format: Number (metres), top unit only</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>What the rock is: descriptive words, then the rock name.
-Format: Text; several lithologies separated by ;</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Lesser lithologies within the unit.
-Format: Text, same format as lithology</t>
+        <t>"y" if the unit is covered: present but not exposed. Its lithology is then your best inference (e.g. shale for a recessive interval).
+Format: y, or blank</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -755,7 +655,7 @@
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>Age at the top. Usually blank: it is taken from the unit above. Fill only on the top unit if its age is known.
+        <t>Age at the top. Usually blank: it is taken from the unit above. Fill only on the top unit if its age is known, or give the empty closing row a b_int instead.
 Format: Interval name, or blank</t>
       </text>
     </comment>
@@ -779,7 +679,119 @@
     </comment>
     <comment ref="Q1" authorId="0" shapeId="0">
       <text>
-        <t>Generalizations, gaps or covered intervals, anything a reader should know.
+        <t>Generalizations, gaps, anything a reader should know.
+Format: Text</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Macrostrat</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Which column this unit belongs to.
+Format: A col_id from the columns tab</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Leave blank if the column is one continuous section. Use a new ID only where the age model breaks (e.g. a fault).
+Format: Text, or blank</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>HEIGHT OF THE BOTTOM of this unit, in metres measured up from the base of the column (base = 0). Every unit needs one.
+Format: Number (metres)</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>HEIGHT OF THE TOP of this unit. Fill it ONLY on the topmost unit of each column, or on a unit below a gap; every other top is taken from the b_pos of the unit above. Or leave it blank and add an empty closing row above the top unit, with only col_id and b_pos.
+Format: Number (metres), top unit or below a gap</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>What the rock is: descriptive words, then the rock name.
+Format: Text; several lithologies separated by ;</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Lesser lithologies within the unit.
+Format: Text, same format as lithology</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>"y" if the unit is covered: present but not exposed. Its lithology is then your best inference (e.g. shale for a recessive interval).
+Format: y, or blank</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Formation or member name, as named in Macrostrat. Fill strat_name, unit_name, or both: each unit needs at least one. If unit_name is blank, this becomes the unit's name.
+Format: Text</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>A local name for the unit (e.g. "upper carbonate"). Fill unit_name, strat_name, or both: each unit needs at least one. If both are filled, this is the unit's name.
+Format: Text</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Type of contact at the bottom of the unit.
+Format: Text, e.g. nonconformity, conformable</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>AGE AT THE BOTTOM of this unit, as a geologic time interval. Fill only at tie points (where you know the age); at least 2 per column. Ages in between are interpolated.
+Format: Macrostrat interval name (use the dropdown)</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>WHERE IN THAT INTERVAL the bottom falls: 0 = start (oldest) of the interval, 0.5 = middle, 1 = end (youngest). A blank counts as 0, so give a best guess.
+Format: Number from 0 to 1</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>Age at the top. Usually blank: it is taken from the unit above. Fill only on the top unit if its age is known, or give the empty closing row a b_int instead.
+Format: Interval name, or blank</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>Where in t_int the top falls (0-1). Usually blank.
+Format: Number 0-1, or blank</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>Why you chose each age tie point and proportion.
+Format: Text</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional label linking to the facies tab. Not read on upload: still fill lithology.
+Format: Text, e.g. F1</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>Generalizations, gaps, anything a reader should know.
 Format: Text</t>
       </text>
     </comment>
@@ -1117,7 +1129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1287,7 +1299,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>One row per unit. A: heights (b_pos = bottom of the unit in metres above the column base; t_pos = top, on the topmost unit only). B: rock (lithology, plus strat_name and/or unit_name). C: ages at tie points (b_int + b_prop).</t>
+          <t>One row per unit. A: heights (b_pos = bottom of the unit in metres above the column base; t_pos = top, on the topmost unit or below a gap, or end with an empty closing row holding only b_pos). B: rock (lithology, plus strat_name and/or unit_name). C: ages at tie points (b_int + b_prop).</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1359,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Every column has a top unit with t_pos and at least 2 age tie points (b_int + b_prop).</t>
+          <t>Every column has a top (t_pos on the top unit, or an empty closing row with only b_pos) and at least 2 age tie points (b_int + b_prop).</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1433,7 @@
     <row r="31" ht="32" customHeight="1">
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Units can be in any order; the ingester sorts them by b_pos. The top of each unit is taken from the base of the unit above.</t>
+          <t>Units can be in any order; the ingester sorts them by b_pos. The top of each unit is taken from the base of the unit above. The topmost unit's top is its own t_pos, or an empty closing row above it holding only col_id and b_pos.</t>
         </is>
       </c>
     </row>
@@ -1442,19 +1454,26 @@
     <row r="34" ht="32" customHeight="1">
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Gaps or covered intervals: add them as a unit with no lithology and explain in comments.</t>
+          <t>Covered intervals: add them as a unit with covered = y, and give your best inference of the lithology.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="32" customHeight="1">
       <c r="B35" s="2" t="inlineStr">
         <is>
+          <t>Gaps (missing rock): give the unit below the gap its own t_pos, and explain in comments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="B36" s="2" t="inlineStr">
+        <is>
           <t>Extra tabs (this one, the example tabs, facies and interval_names) are ignored on upload.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B24:C24"/>
@@ -1465,6 +1484,7 @@
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B26:C26"/>
@@ -14169,7 +14189,7 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>"y" = a blank lithology/strat_name/etc. cell copies the value from the unit above (type "none" to stop). Do not leave blank.</t>
+          <t>"y" = a blank lithology/strat_name/etc. cell copies the value from the unit below it, so enter a value at the base of the interval it applies to (type "none" to stop). Do not leave blank.</t>
         </is>
       </c>
       <c r="D9" s="26" t="inlineStr">
@@ -14546,7 +14566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14555,16 +14575,17 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14598,61 +14619,66 @@
           <t>minor_lith</t>
         </is>
       </c>
-      <c r="G1" s="27" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>covered</t>
+        </is>
+      </c>
+      <c r="H1" s="27" t="inlineStr">
         <is>
           <t>strat_name</t>
         </is>
       </c>
-      <c r="H1" s="27" t="inlineStr">
+      <c r="I1" s="27" t="inlineStr">
         <is>
           <t>unit_name</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>basal_surface</t>
         </is>
       </c>
-      <c r="J1" s="28" t="inlineStr">
+      <c r="K1" s="28" t="inlineStr">
         <is>
           <t>b_int</t>
         </is>
       </c>
-      <c r="K1" s="28" t="inlineStr">
+      <c r="L1" s="28" t="inlineStr">
         <is>
           <t>b_prop</t>
         </is>
       </c>
-      <c r="L1" s="28" t="inlineStr">
+      <c r="M1" s="28" t="inlineStr">
         <is>
           <t>t_int</t>
         </is>
       </c>
-      <c r="M1" s="28" t="inlineStr">
+      <c r="N1" s="28" t="inlineStr">
         <is>
           <t>t_prop</t>
         </is>
       </c>
-      <c r="N1" s="11" t="inlineStr">
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>age_model_notes</t>
         </is>
       </c>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>facies</t>
         </is>
       </c>
-      <c r="P1" s="11" t="inlineStr">
+      <c r="Q1" s="11" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:H2000">
+  <conditionalFormatting sqref="H2:I2000">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND($A2&lt;&gt;"",$G2="",$H2="")</formula>
+      <formula>AND($A2&lt;&gt;"",$H2="",$I2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="7">
@@ -14662,20 +14688,20 @@
     <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="Bottom of the unit, metres above column base" type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>-100000</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="Top of the unit - topmost unit only" type="decimal" errorStyle="stop" operator="greaterThan">
+    <dataValidation sqref="D2:D2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="Top of the unit - topmost unit or below a gap" type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>-100000</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="Pick a Macrostrat interval name" type="list" errorStyle="warning">
+    <dataValidation sqref="K2:K2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="Pick a Macrostrat interval name" type="list" errorStyle="warning">
       <formula1>=interval_names!$A$2:$A$1716</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="0 = oldest end, 1 = youngest end" type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="L2:L2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="0 = oldest end, 1 = youngest end" type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="L2:L2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="Pick a Macrostrat interval name" type="list" errorStyle="warning">
+    <dataValidation sqref="M2:M2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="Pick a Macrostrat interval name" type="list" errorStyle="warning">
       <formula1>=interval_names!$A$2:$A$1716</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="0-1" type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="N2:N2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="0-1" type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -14692,7 +14718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -14702,16 +14728,17 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14746,52 +14773,57 @@
           <t>minor_lith</t>
         </is>
       </c>
-      <c r="H1" s="27" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>covered</t>
+        </is>
+      </c>
+      <c r="I1" s="27" t="inlineStr">
         <is>
           <t>strat_name</t>
         </is>
       </c>
-      <c r="I1" s="27" t="inlineStr">
+      <c r="J1" s="27" t="inlineStr">
         <is>
           <t>unit_name</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>basal_surface</t>
         </is>
       </c>
-      <c r="K1" s="28" t="inlineStr">
+      <c r="L1" s="28" t="inlineStr">
         <is>
           <t>b_int</t>
         </is>
       </c>
-      <c r="L1" s="28" t="inlineStr">
+      <c r="M1" s="28" t="inlineStr">
         <is>
           <t>b_prop</t>
         </is>
       </c>
-      <c r="M1" s="28" t="inlineStr">
+      <c r="N1" s="28" t="inlineStr">
         <is>
           <t>t_int</t>
         </is>
       </c>
-      <c r="N1" s="28" t="inlineStr">
+      <c r="O1" s="28" t="inlineStr">
         <is>
           <t>t_prop</t>
         </is>
       </c>
-      <c r="O1" s="11" t="inlineStr">
+      <c r="P1" s="11" t="inlineStr">
         <is>
           <t>age_model_notes</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>facies</t>
         </is>
       </c>
-      <c r="Q1" s="11" t="inlineStr">
+      <c r="R1" s="11" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
@@ -14820,7 +14852,7 @@
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>HEIGHT OF THE TOP of this unit. Fill it ONLY on the topmost unit of each column; every other top is taken from the b_pos of the unit above.</t>
+          <t>HEIGHT OF THE TOP of this unit. Fill it ONLY on the topmost unit of each column, or on a unit below a gap; every other top is taken from the b_pos of the unit above. Or leave it blank and add an empty closing row above the top unit, with only col_id and b_pos.</t>
         </is>
       </c>
       <c r="F2" s="15" t="inlineStr">
@@ -14835,52 +14867,57 @@
       </c>
       <c r="H2" s="15" t="inlineStr">
         <is>
+          <t>"y" if the unit is covered: present but not exposed. Its lithology is then your best inference (e.g. shale for a recessive interval).</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
           <t>Formation or member name, as named in Macrostrat. Fill strat_name, unit_name, or both: each unit needs at least one. If unit_name is blank, this becomes the unit's name.</t>
         </is>
       </c>
-      <c r="I2" s="15" t="inlineStr">
+      <c r="J2" s="15" t="inlineStr">
         <is>
           <t>A local name for the unit (e.g. "upper carbonate"). Fill unit_name, strat_name, or both: each unit needs at least one. If both are filled, this is the unit's name.</t>
         </is>
       </c>
-      <c r="J2" s="15" t="inlineStr">
+      <c r="K2" s="15" t="inlineStr">
         <is>
           <t>Type of contact at the bottom of the unit.</t>
         </is>
       </c>
-      <c r="K2" s="15" t="inlineStr">
+      <c r="L2" s="15" t="inlineStr">
         <is>
           <t>AGE AT THE BOTTOM of this unit, as a geologic time interval. Fill only at tie points (where you know the age); at least 2 per column. Ages in between are interpolated.</t>
         </is>
       </c>
-      <c r="L2" s="15" t="inlineStr">
+      <c r="M2" s="15" t="inlineStr">
         <is>
           <t>WHERE IN THAT INTERVAL the bottom falls: 0 = start (oldest) of the interval, 0.5 = middle, 1 = end (youngest). A blank counts as 0, so give a best guess.</t>
         </is>
       </c>
-      <c r="M2" s="15" t="inlineStr">
-        <is>
-          <t>Age at the top. Usually blank: it is taken from the unit above. Fill only on the top unit if its age is known.</t>
-        </is>
-      </c>
       <c r="N2" s="15" t="inlineStr">
         <is>
+          <t>Age at the top. Usually blank: it is taken from the unit above. Fill only on the top unit if its age is known, or give the empty closing row a b_int instead.</t>
+        </is>
+      </c>
+      <c r="O2" s="15" t="inlineStr">
+        <is>
           <t>Where in t_int the top falls (0-1). Usually blank.</t>
         </is>
       </c>
-      <c r="O2" s="15" t="inlineStr">
+      <c r="P2" s="15" t="inlineStr">
         <is>
           <t>Why you chose each age tie point and proportion.</t>
         </is>
       </c>
-      <c r="P2" s="15" t="inlineStr">
+      <c r="Q2" s="15" t="inlineStr">
         <is>
           <t>Optional label linking to the facies tab. Not read on upload: still fill lithology.</t>
         </is>
       </c>
-      <c r="Q2" s="15" t="inlineStr">
-        <is>
-          <t>Generalizations, gaps or covered intervals, anything a reader should know.</t>
+      <c r="R2" s="15" t="inlineStr">
+        <is>
+          <t>Generalizations, gaps, anything a reader should know.</t>
         </is>
       </c>
     </row>
@@ -14907,7 +14944,7 @@
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>Number (metres), top unit only</t>
+          <t>Number (metres), top unit or below a gap</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
@@ -14922,50 +14959,55 @@
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
+          <t>y, or blank</t>
+        </is>
+      </c>
+      <c r="I3" s="16" t="inlineStr">
+        <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="I3" s="16" t="inlineStr">
+      <c r="J3" s="16" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="J3" s="16" t="inlineStr">
+      <c r="K3" s="16" t="inlineStr">
         <is>
           <t>Text, e.g. nonconformity, conformable</t>
         </is>
       </c>
-      <c r="K3" s="16" t="inlineStr">
+      <c r="L3" s="16" t="inlineStr">
         <is>
           <t>Macrostrat interval name (use the dropdown)</t>
         </is>
       </c>
-      <c r="L3" s="16" t="inlineStr">
+      <c r="M3" s="16" t="inlineStr">
         <is>
           <t>Number from 0 to 1</t>
         </is>
       </c>
-      <c r="M3" s="16" t="inlineStr">
+      <c r="N3" s="16" t="inlineStr">
         <is>
           <t>Interval name, or blank</t>
         </is>
       </c>
-      <c r="N3" s="16" t="inlineStr">
+      <c r="O3" s="16" t="inlineStr">
         <is>
           <t>Number 0-1, or blank</t>
         </is>
       </c>
-      <c r="O3" s="16" t="inlineStr">
+      <c r="P3" s="16" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="P3" s="16" t="inlineStr">
+      <c r="Q3" s="16" t="inlineStr">
         <is>
           <t>Text, e.g. F1</t>
         </is>
       </c>
-      <c r="Q3" s="16" t="inlineStr">
+      <c r="R3" s="16" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
@@ -14995,24 +15037,25 @@
         </is>
       </c>
       <c r="G4" s="18" t="n"/>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H4" s="18" t="n"/>
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>Wood Canyon Formation</t>
         </is>
       </c>
-      <c r="I4" s="18" t="n"/>
       <c r="J4" s="18" t="n"/>
       <c r="K4" s="18" t="n"/>
       <c r="L4" s="18" t="n"/>
       <c r="M4" s="18" t="n"/>
       <c r="N4" s="18" t="n"/>
       <c r="O4" s="18" t="n"/>
-      <c r="P4" s="18" t="inlineStr">
+      <c r="P4" s="18" t="n"/>
+      <c r="Q4" s="18" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="Q4" s="19" t="inlineStr">
+      <c r="R4" s="19" t="inlineStr">
         <is>
           <t>Top of measured section, so t_pos is filled.</t>
         </is>
@@ -15040,24 +15083,25 @@
         </is>
       </c>
       <c r="G5" s="18" t="n"/>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>Wood Canyon Formation</t>
         </is>
       </c>
-      <c r="I5" s="18" t="n"/>
       <c r="J5" s="18" t="n"/>
       <c r="K5" s="18" t="n"/>
       <c r="L5" s="18" t="n"/>
       <c r="M5" s="18" t="n"/>
       <c r="N5" s="18" t="n"/>
       <c r="O5" s="18" t="n"/>
-      <c r="P5" s="18" t="inlineStr">
+      <c r="P5" s="18" t="n"/>
+      <c r="Q5" s="18" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="Q5" s="19" t="inlineStr">
+      <c r="R5" s="19" t="inlineStr">
         <is>
           <t>Top comes from the unit above (6.16 m).</t>
         </is>
@@ -15085,24 +15129,25 @@
         </is>
       </c>
       <c r="G6" s="18" t="n"/>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="18" t="inlineStr">
         <is>
           <t>Wood Canyon Formation</t>
         </is>
       </c>
-      <c r="I6" s="18" t="n"/>
       <c r="J6" s="18" t="n"/>
       <c r="K6" s="18" t="n"/>
       <c r="L6" s="18" t="n"/>
       <c r="M6" s="18" t="n"/>
       <c r="N6" s="18" t="n"/>
       <c r="O6" s="18" t="n"/>
-      <c r="P6" s="18" t="inlineStr">
+      <c r="P6" s="18" t="n"/>
+      <c r="Q6" s="18" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="Q6" s="18" t="n"/>
+      <c r="R6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
@@ -15126,34 +15171,35 @@
         </is>
       </c>
       <c r="G7" s="18" t="n"/>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="18" t="inlineStr">
         <is>
           <t>Wood Canyon Formation</t>
         </is>
       </c>
-      <c r="I7" s="18" t="n"/>
       <c r="J7" s="18" t="n"/>
-      <c r="K7" s="18" t="inlineStr">
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="inlineStr">
         <is>
           <t>Terreneuvian</t>
         </is>
       </c>
-      <c r="L7" s="18" t="n">
+      <c r="M7" s="18" t="n">
         <v>0.75</v>
       </c>
-      <c r="M7" s="18" t="n"/>
       <c r="N7" s="18" t="n"/>
-      <c r="O7" s="19" t="inlineStr">
+      <c r="O7" s="18" t="n"/>
+      <c r="P7" s="19" t="inlineStr">
         <is>
           <t>Placeholder age: base and datum tied within the Terreneuvian; proportions are best guesses.</t>
         </is>
       </c>
-      <c r="P7" s="18" t="inlineStr">
+      <c r="Q7" s="18" t="inlineStr">
         <is>
           <t>F2</t>
         </is>
       </c>
-      <c r="Q7" s="19" t="inlineStr">
+      <c r="R7" s="19" t="inlineStr">
         <is>
           <t>Datum bed: age tie point, same b_int/b_prop in every column.</t>
         </is>
@@ -15181,38 +15227,39 @@
         </is>
       </c>
       <c r="G8" s="18" t="n"/>
-      <c r="H8" s="18" t="inlineStr">
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="18" t="inlineStr">
         <is>
           <t>Wood Canyon Formation</t>
         </is>
       </c>
-      <c r="I8" s="18" t="n"/>
-      <c r="J8" s="18" t="inlineStr">
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="18" t="inlineStr">
         <is>
           <t>nonconformity</t>
         </is>
       </c>
-      <c r="K8" s="18" t="inlineStr">
+      <c r="L8" s="18" t="inlineStr">
         <is>
           <t>Terreneuvian</t>
         </is>
       </c>
-      <c r="L8" s="18" t="n">
+      <c r="M8" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="M8" s="18" t="n"/>
       <c r="N8" s="18" t="n"/>
-      <c r="O8" s="19" t="inlineStr">
+      <c r="O8" s="18" t="n"/>
+      <c r="P8" s="19" t="inlineStr">
         <is>
           <t>Placeholder age: base and datum tied within the Terreneuvian; proportions are best guesses.</t>
         </is>
       </c>
-      <c r="P8" s="18" t="inlineStr">
+      <c r="Q8" s="18" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="Q8" s="19" t="inlineStr">
+      <c r="R8" s="19" t="inlineStr">
         <is>
           <t>Base of column (b_pos = 0): age tie point.</t>
         </is>

</xml_diff>